<commit_message>
Rebuild Mode 1 Golden Path doc with fresh Playwright run on mbx-ee-dev
New dedicated test material ("E2E Mode1 Fresh Test") instead of reusing
"Rosso Levanto Test", which still carried a leftover FIFO cost layer from
the Mode 3 fixture's block (BLK-26-0013) — reusing it produced a wrong
COGS (40,000 instead of 30,000) on the first attempt. Fresh fixture:
PO P00048 -> BLK-26-0023 -> BILL/2026/09/0003 -> SO S00120 ->
EG01/OUT/00074 -> INV/2026/00024. Archived-doc entry added linking back
to the old v2 doc, now moved under qa/_archive/.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/client-docs/test-cases/emg-o-test-cases-e2e-mode1.xlsx
+++ b/client-docs/test-cases/emg-o-test-cases-e2e-mode1.xlsx
@@ -704,15 +704,15 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>Vendor = "Demo Supplier - Global Stone Quarry"
-สินค้า = SY-TST-Onyx-Rosa - Block
+          <t>Vendor = "ทดสอบ E2E - Test Quarry Vendor"
+สินค้า = E2E Mode1 Fresh Test - Block
 จำนวน = 2.00 m³
 ราคา/หน่วย = 15,000</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>PO ยืนยันสำเร็จ (state = Purchase Order) ยอดรวมคำนวณถูกต้อง (จำนวน × ราคา + VAT) — ตัวอย่างจริงที่ทดสอบ: P00052 ยอดรวม 32,100.00</t>
+          <t>PO ยืนยันสำเร็จ (state = Purchase Order) ยอดรวมคำนวณถูกต้อง (จำนวน × ราคา + VAT) — ตัวอย่างจริงที่ทดสอบ: P00048 ยอดรวม 32,100.00</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -758,7 +758,7 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>บันทึกสำเร็จ ได้เลขก้อนอัตโนมัติ (ตัวอย่างจริง: BLK-26-0068) ช่อง "PO Cost / CBM" ขึ้น 15,000 ให้เอง, "Sales Price / CBM" ขึ้น 17,500 ให้เองจาก List Price ของ Block Product, Remaining CBM = 2.00 (รับสต๊อกเข้าจริงแล้ว)</t>
+          <t>บันทึกสำเร็จ ได้เลขก้อนอัตโนมัติ (ตัวอย่างจริง: BLK-26-0023) ช่อง "PO Cost / CBM" ขึ้น 15,000 ให้เอง, "Sales Price / CBM" ขึ้น 17,500 ให้เองจาก List Price ของ Block Product, Remaining CBM = 2.00 (รับสต๊อกเข้าจริงแล้ว)</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -768,7 +768,7 @@
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>✨ ใหม่ (2026-09-09): ไม่ต้องเปิด Inventory &gt; Blocks &gt; New แล้วไปหา PO Line เองอีกต่อไป — กดปุ่มนี้ตรงบรรทัด PO ได้เลย ระบบกรอก Material/Supplier/Warehouse/Total CBM ให้อัตโนมัติจากบรรทัดนั้น ยังคงไม่มีขั้นตอน "Validate Receipt" แยกต่างหาก — Receipt ที่ระบบสร้างให้อัตโนมัติจาก PO จะถูกยกเลิกให้เองเบื้องหลัง (กันสต๊อกซ้ำ) ไม่ต้องไปกดอะไรกับมัน</t>
+          <t>กดปุ่มนี้ตรงบรรทัด PO ได้เลย ไม่ต้องเปิด Inventory &gt; Blocks &gt; New แล้วไปหา PO Line เอง ระบบกรอก Material/Supplier/Warehouse/Total CBM ให้อัตโนมัติจากบรรทัดนั้น ไม่มีขั้นตอน "Validate Receipt" แยกต่างหาก — Receipt ที่ระบบสร้างให้อัตโนมัติจาก PO จะถูกยกเลิกให้เองเบื้องหลัง (กันสต๊อกซ้ำ) ไม่ต้องไปกดอะไรกับมัน</t>
         </is>
       </c>
       <c r="I5" s="7" t="n"/>
@@ -803,13 +803,13 @@
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>Vendor = "Demo Supplier - Global Stone Quarry"
-Auto-Complete = P00052</t>
+          <t>Vendor = "ทดสอบ E2E - Test Quarry Vendor"
+Auto-Complete = P00048</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>บิลสถานะ Posted ยอดตรงกับ PO บัญชีที่ลงถูกต้องเป็น "113110 Inventory - Stone Blocks (Raw)" ไม่ใช่บัญชี COGS ทั่วไป (ตัวอย่างจริง: BILL/2026/09/0002, 32,100.00)</t>
+          <t>บิลสถานะ Posted ยอดตรงกับ PO บัญชีที่ลงถูกต้องเป็น "113110 Inventory - Stone Blocks (Raw)" ไม่ใช่บัญชี COGS ทั่วไป (ตัวอย่างจริง: BILL/2026/09/0003, 32,100.00)</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -948,8 +948,8 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>ลูกค้า = "E2E Test Customer"
-สินค้า = SY-TST-Onyx-Rosa - Block</t>
+          <t>ลูกค้า = "ทดสอบ E2E - Test Customer"
+สินค้า = E2E Mode1 Fresh Test - Block</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
@@ -987,18 +987,18 @@
       <c r="D5" s="7" t="inlineStr">
         <is>
           <t>1. กดปุ่ม "Sell Whole Block" บนบรรทัด
-2. หน้าต่าง "Select Block" เลือก Block ที่ซื้อไว้ (เช่น BLK-26-0068)
+2. หน้าต่าง "Select Block" เลือก Block ที่ซื้อไว้ (เช่น BLK-26-0023)
 3. กด "Confirm Selection"</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>เลือก Block = BLK-26-0068</t>
+          <t>เลือก Block = BLK-26-0023</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>บรรทัด SO ปรับจำนวนเป็น CBM ทั้งหมดของก้อนนั้นอัตโนมัติ (2.00) ราคาต่อหน่วยเปลี่ยนเป็น 17,500.00 ทันที (จาก Sales Price / CBM ของก้อน ไม่ใช่ราคาที่พิมพ์ไว้ก่อนหน้า) ยอดรวมบรรทัด 35,000.00</t>
+          <t>บรรทัด SO ปรับจำนวนเป็น CBM ทั้งหมดของก้อนนั้นอัตโนมัติ (2.00) ราคาต่อหน่วยเปลี่ยนเป็น 17,500.00 ทันที (จาก Sales Price / CBM ของก้อน) ยอดรวมบรรทัด 35,000.00</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>✨ ใหม่ (2026-09-09): เดิม Unit Price ต้องพิมพ์เองหลังเลือกก้อน ตอนนี้ระบบดึง "Sales Price / CBM" ของก้อนนั้นมาใส่ให้อัตโนมัติทันทีที่กด Confirm Selection — พิมพ์ราคาอื่นทับไว้ก่อนก็ได้ ระบบจะเขียนทับด้วยราคาจริงของก้อนเสมอ</t>
+          <t>ระบบดึง "Sales Price / CBM" ของก้อนนั้นมาใส่ให้อัตโนมัติทันทีที่กด Confirm Selection — พิมพ์ราคาอื่นทับไว้ก่อนก็ได้ ระบบจะเขียนทับด้วยราคาจริงของก้อนเสมอ</t>
         </is>
       </c>
       <c r="I5" s="7" t="n"/>
@@ -1044,7 +1044,7 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>SO เปลี่ยนสถานะเป็น Sales Order มี Delivery Order เกิดขึ้นให้อัตโนมัติ 1 ใบ (ตัวอย่างจริง: S00091 → EG01/OUT/00067)</t>
+          <t>SO เปลี่ยนสถานะเป็น Sales Order มี Delivery Order เกิดขึ้นให้อัตโนมัติ 1 ใบ (ตัวอย่างจริง: S00120 → EG01/OUT/00074)</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -1374,7 +1374,7 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>ใบส่งของเปลี่ยนสถานะเป็น Done (ตัวอย่างจริง: EG01/OUT/00067) — Block ก้อนนั้นหายจากสต๊อกที่ขายได้ (Available) แล้ว</t>
+          <t>ใบส่งของเปลี่ยนสถานะเป็น Done (ตัวอย่างจริง: EG01/OUT/00074) — Block ก้อนนั้นหายจากสต๊อกที่ขายได้ (Available) แล้ว</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -1518,7 +1518,7 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>ใบแจ้งหนี้สถานะ Posted ยอดรวมตรงกับ SO รวม VAT (ตัวอย่างจริง: INV/2026/00003, 37,450.00)</t>
+          <t>ใบแจ้งหนี้สถานะ Posted ยอดรวมตรงกับ SO รวม VAT (ตัวอย่างจริง: INV/2026/00024, 37,450.00)</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -1602,7 +1602,7 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>เห็น 5 บรรทัดบนใบแจ้งหนี้ใบเดียว: เครดิต 411110 Sales Revenue - Block Direct Sale (Mode 1), เดบิต 113110 Inventory (ตัดออก), เดบิต 511110 COGS - Block Direct Sale (Mode 1), เครดิต 213200 Output VAT, เดบิต 112100 Trade Receivables — ตัวอย่างจริง: รายได้ 35,000 / COGS-Inventory คู่ละ 30,000 / VAT 2,450 / ลูกหนี้ 37,450 (ยอดรวมสมดุล 67,450 = 67,450)</t>
+          <t>เห็น 5 บรรทัดบนใบแจ้งหนี้ใบเดียว: เครดิต 411110 Sales Revenue - Block Direct Sale (Mode 1), เดบิต 113110 Inventory (ตัดออก), เดบิต 511110 COGS - Stone Sales (all modes), เครดิต 213200 Output VAT, เดบิต 112100 Trade Receivables — ตัวอย่างจริง: รายได้ 35,000 / COGS-Inventory คู่ละ 30,000 / VAT 2,450 / ลูกหนี้ 37,450 (ยอดรวมสมดุล 67,450 = 67,450)</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -1635,7 +1635,7 @@
       <c r="D7" s="7" t="inlineStr">
         <is>
           <t>1. เปิด Accounting &gt; Journal Entries
-2. ค้นหา entry ที่มี Reference ตรงกับเลขที่ใบส่งของ (เช่น EG01/OUT/00067)</t>
+2. ค้นหา entry ที่มี Reference ตรงกับเลขที่ใบส่งของ (เช่น EG01/OUT/00074)</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -1645,7 +1645,7 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>ไม่พบ Journal Entry แยกต่างหากสำหรับใบส่งของนี้เลย — COGS/Inventory มีบันทึกอยู่ที่เดียวคือในใบแจ้งหนี้ (INV/2026/00003) ไม่มีการนับซ้ำ</t>
+          <t>ไม่พบ Journal Entry แยกต่างหากสำหรับใบส่งของนี้เลย — COGS/Inventory มีบันทึกอยู่ที่เดียวคือในใบแจ้งหนี้ (INV/2026/00024) ไม่มีการนับซ้ำ</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
@@ -1655,7 +1655,7 @@
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>✅ ปิดเคสแล้ว — ตรวจซ้ำด้วย fixture ใหม่ (2026-09-09) ยืนยันว่าการแก้ไข ADR-054/055 (session ก่อนหน้า) ยังใช้ได้ดี: ไม่มี Journal Entry แยกต่างหากจากใบส่งของอีกต่อไป (เดิมมีปัญหาชื่อขึ้นต้น STJ ซ้ำกับใบแจ้งหนี้) — Delivery ไม่สร้าง Journal Entry ของตัวเองแล้ว COGS มีบันทึกอยู่ที่เดียวคือในใบแจ้งหนี้ (TC-E2E-M1-11)</t>
+          <t>✅ ตรวจซ้ำด้วย fixture ใหม่ทั้งชุด (2026-09-14, วัสดุใหม่ล้วนๆ) ยืนยันว่าการแก้ไข ADR-054/055 ยังใช้ได้ดี: ไม่มี Journal Entry แยกต่างหากจากใบส่งของอีกต่อไป COGS มีบันทึกอยู่ที่เดียวคือในใบแจ้งหนี้ (TC-E2E-M1-11) — ตรวจแล้วไม่มี STJ entry อ้างอิงถึง EG01/OUT/00074 เลย</t>
         </is>
       </c>
       <c r="I7" s="7" t="n"/>
@@ -1840,7 +1840,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>E7. ต้นทุนแยกตามมิติ (Cost-by-Material Analytics) — Analytic-Architecture ใหม่ 2026-09-09</t>
+          <t>E7. ต้นทุนแยกตามมิติ (Cost-by-Material Analytics) — Analytic-Architecture 3 มิติ</t>
         </is>
       </c>
     </row>
@@ -1935,7 +1935,7 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>เห็น 2 ป้ายบนบรรทัดเดียว: "Marble | SY-TST-Onyx-Rosa" (หมวดวัสดุ+วัสดุ) และ "BLK-26-0068" (ก้อนนี้โดยเฉพาะ) — ไม่ต้องตั้งค่าเอง ระบบแท็กให้ตั้งแต่กด Sell Whole Block</t>
+          <t>เห็น 3 ป้ายบนบรรทัดเดียว: "E2E Mode1 Fresh Test" (วัสดุ), "BLK-26-0023" (ก้อนนี้โดยเฉพาะ), และ "Marble" (หมวดวัสดุ) — ไม่ต้องตั้งค่าเอง ระบบแท็กให้ตั้งแต่กด Sell Whole Block</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -1945,7 +1945,7 @@
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>✨ ใหม่ (2026-09-09): ทุกบรรทัดที่ผูกกับ Block จะถูกแท็กเข้า 3 มิติพร้อมกันโดยอัตโนมัติ — Block (ก้อนนี้โดยเฉพาะ), หมวดวัสดุ (เช่น Marble ใช้ร่วมกันได้ทุก Marble), และวัสดุ (เฉพาะ SY-TST-Onyx-Rosa) ไม่ต้องพิมพ์เอง ทำให้ดูกำไร/ต้นทุนแยกได้ทั้งรายก้อน รายหมวดวัสดุ หรือรายวัสดุเป๊ะๆ</t>
+          <t>ทุกบรรทัดที่ผูกกับ Block จะถูกแท็กเข้า 3 มิติพร้อมกันโดยอัตโนมัติ — Block (ก้อนนี้โดยเฉพาะ), หมวดวัสดุ (เช่น Marble ใช้ร่วมกันได้ทุก Marble), และวัสดุ (เฉพาะ E2E Mode1 Fresh Test) ไม่ต้องพิมพ์เอง ทำให้ดูกำไร/ต้นทุนแยกได้ทั้งรายก้อน รายหมวดวัสดุ หรือรายวัสดุเป๊ะๆ</t>
         </is>
       </c>
       <c r="I4" s="7" t="n"/>

</xml_diff>